<commit_message>
Show the Senna coins and lemonade stills on the lesson 1 scenario beats.
The Explorer workbook image cells for those two beats are the import source. Numbered screens and the intro scene stay as they were.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -711,7 +711,11 @@
 Senna earned it walking dogs in the neighborhood. "It's a great way to make some money," Senna says.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>em1-02-l1r7-senna-coins-r3.webp</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
@@ -878,7 +882,11 @@
 He decides to start his own business: a lemonade stand!</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>em1-03-l1r11-lars-lemonade-r3.webp</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>

</xml_diff>

<commit_message>
Show the bike-note still on the lesson 2 scenario beat.
The intro lemonade scene and the numbered lesson screens stay unchanged.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -1262,7 +1262,11 @@
 Mom says she'll help, but Lars has to pay for part of it himself. Pocket money won't get him there, so Lars makes a plan: a lemonade stand!</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>em1-04-l2r20-lars-mom-bike-note-r3.webp</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add Explorer batch 3 art and place the two stills that match story beats.
The other files are in the pairs folder with no workbook row, because those sheet rows are not story beats or the text does not match the picture.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -2934,7 +2934,11 @@
 "I could design the sign for your stand," she says.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n"/>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l6-r1.webp</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="inlineStr">
@@ -3414,7 +3418,11 @@
 His startup envelope stays at home. Today's money is just for the mall.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="n"/>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l7-r1.webp</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="n"/>
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Place Explorer batch 3 stills by story-beat text.
Clear the held lemon-ticket beat and leave the locked intro and em1 stills as they are.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -1300,7 +1300,11 @@
 Mom agrees, as long as the stand goes by their front gate, where she can see him.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-stand-set-r1.webp</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="inlineStr">
@@ -1548,7 +1552,11 @@
 Every time he gets money, some goes in. Next time something breaks, he'll be ready.</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-emergencies-jar-r1.webp</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
@@ -1717,7 +1725,11 @@
 "Before you buy something, ask if you really want or need it," says his school friend Mason. "That's how I've saved so much."</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-lars-mason-r1.webp</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
@@ -2108,7 +2120,11 @@
           <t>Lars grabs an envelope to keep his stand money separate. He writes 'Startup money needed: $15' on the front.</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-lars-thinking-r1.webp</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="inlineStr">
@@ -2142,7 +2158,11 @@
 He pictures his stand by the front gate, with a bright sign and a jug of lemonade.</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-stand-set-r1.webp</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="n"/>
       <c r="H40" s="2" t="n"/>
       <c r="I40" s="2" t="inlineStr">
@@ -2900,7 +2920,11 @@
 His startup money stayed at $10, and he still has $3 spare.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l6-r1.webp</t>
+        </is>
+      </c>
       <c r="G58" s="2" t="n"/>
       <c r="H58" s="2" t="n"/>
       <c r="I58" s="2" t="inlineStr">
@@ -2934,11 +2958,7 @@
 "I could design the sign for your stand," she says.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l6-r1.webp</t>
-        </is>
-      </c>
+      <c r="F59" s="2" t="n"/>
       <c r="G59" s="2" t="n"/>
       <c r="H59" s="2" t="n"/>
       <c r="I59" s="2" t="inlineStr">
@@ -3009,7 +3029,11 @@
 Mom told the neighbors, and lots of them want to buy lemonade!</t>
         </is>
       </c>
-      <c r="F61" s="2" t="n"/>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l7-r1.webp</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="n"/>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="inlineStr">
@@ -3384,7 +3408,11 @@
 "Deals like that used to get me every time," Lars laughs.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="n"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-slushie-r1.webp</t>
+        </is>
+      </c>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="inlineStr">
@@ -3420,7 +3448,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>beat-ex-m1-l7-r1.webp</t>
+          <t>prop-ex-m1-bike-bubble-r1.webp</t>
         </is>
       </c>
       <c r="G71" s="2" t="n"/>
@@ -3456,7 +3484,11 @@
 What he does with his money today is up to you!</t>
         </is>
       </c>
-      <c r="F72" s="2" t="n"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l8-r2.webp</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="n"/>
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="inlineStr">
@@ -4664,7 +4696,11 @@
 On Saturday, his stand opens by the front gate.</t>
         </is>
       </c>
-      <c r="F101" s="2" t="n"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l9-r1.webp</t>
+        </is>
+      </c>
       <c r="G101" s="2" t="n"/>
       <c r="H101" s="2" t="n"/>
       <c r="I101" s="2" t="inlineStr">
@@ -4697,7 +4733,11 @@
           <t>He's one step closer to his mountain bike!</t>
         </is>
       </c>
-      <c r="F102" s="2" t="n"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-lars-cheering-bike-r1.webp</t>
+        </is>
+      </c>
       <c r="G102" s="2" t="n"/>
       <c r="H102" s="2" t="n"/>
       <c r="I102" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Show the Lesson 5 gelato share still.
The share beat's workbook image cell was empty, so the story slot rendered nothing. It now uses the approved 1600x1200 gelato scene, and every Explorer story beat is checked for a real still.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -2837,7 +2837,11 @@
 His startup envelope still holds $10.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l5-r4.webp</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="n"/>
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Stage Cath's Explorer copy edits for the 18 confirmed cells.
The Lesson 9 close is now one beat before the medal, using the stand still. Choice and sort settings for the gelato share and the movie ideas match the snapshot and still score.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1369,7 +1369,7 @@
       <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Senna loves his new phone case. That night, Lars tells Mom his big dream: swapping his old bike for a better mountain bike.
-Mom says she'll help, but Lars has to pay for part of it himself. Pocket money won't get him there, so Lars makes a plan: a lemonade stand!</t>
+His parents say they'll help, but Lars has to pay for part of it himself. Pocket money won't get him there, so Lars makes a plan.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>First he needs a jug, paper cups, lemons and sugar. That costs money too, so he decides to save for it.
+          <t>Lars wants to run a lemonade stand. First he needs a jug, paper cups, lemons, sugar and ingredients to bake cookies. That all costs money, so he decides to save for it.
 Mom agrees, as long as the stand goes by their front gate, where she can see him.</t>
         </is>
       </c>
@@ -1481,7 +1481,7 @@
       <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Saving for the stand sounds easy. But his friends keep heading to the corner store, and the weeks fly by.
+          <t>Saving for the lemonade stand idea sounds easy, but he keeps spending his money at the corner store. The weeks fly by.
 Then one afternoon, Lars borrows Senna's headphones...</t>
         </is>
       </c>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Over the next few weeks, Lars spends every dollar on fun stuff and forgets to save. Then he breaks Senna's headphones by accident. What's the real problem?</t>
+          <t>He accidentally breaks Senna's headphones. What's the problem Lars faces?</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Lars's friends are all buying a game skin before the timer runs out. Mason sees Lars holding off. What is Lars really doing by waiting?</t>
+          <t>Lars's friends are all buying the game skin before the timer runs out. Mason sees that Lars is holding off. What is Lars really doing by waiting?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2340,7 +2340,7 @@
       <c r="D45" s="2" t="n"/>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Lars grabs an envelope to keep his stand money separate. He writes 'Startup money needed: $15' on the front.</t>
+          <t>Lars grabs an envelope to keep the money for his lemonade stand separate. He writes 'Startup money needed: $15' on the front.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>A birthday gelato costs $5. The only money Lars has is his $10 startup money. What should he do?</t>
+          <t>The gelato costs $5. The only money Lars has is his $10 startup money. What should he do?</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>CHOICE A: 🤝 Skip his own gelato and share Mia's.
+          <t>CHOICE A: 🤝 Skip his own gelato and ask if Mia wants to share.
 CHOICE B: 🍦 Buy his own, because the deal ends today.
 CORRECT: A</t>
         </is>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>True or false: the gelato is a need because the deal is only on today.</t>
+          <t>True or false: the gelato is a 'Need' because the deal is only on today.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>At the counter, a sign flashes: DEAL ENDS TODAY! Lars feels left out without his own cup. What should he do now?</t>
+          <t>The birthday deal is only on today. Lars feels left out without his own cup. What should he do now?</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Earlier this week, Lars nearly bought a $5 mini dart blaster. What would have happened if he had bought it?</t>
+          <t>Earlier this week, Lars nearly bought a $5 mini dart blaster, but he decided he didn't need it. What would have happened if he had bought it?</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -3041,7 +3041,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Lars has $8, and his half of the movie costs $5. Which ideas work without going below zero or borrowing? Sort each idea into Yes or No.</t>
+          <t>Because he didn't buy the blaster, Lars has $8. His half of the movie costs $5. Which are good ideas for Lars? Sort each idea into Yes or No.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -3053,8 +3053,8 @@
         <is>
           <t>ITEMS:
 YES: 🎟️ Pay his $5 half
-YES: 💰 Keep $3 for later
-NO: 🎯 Dart blaster and the movie
+YES: 💰 Save the remaining $3 for later
+NO: 🎯 Buy the dart blaster and movie ticket
 NO: 🙋 Borrow $5 from Senna</t>
         </is>
       </c>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Mom will pay half of the $10. Lars will pay his $5 from his $8. How much will he have left?</t>
+          <t>Lars's parents will pay half of the $10. Lars pays the other half from the $8 he has. How much will Lars have left?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -3407,8 +3407,8 @@
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>At the bus stop, Lars tells Mason his big news.
-Mom told the neighbors, and lots of them want to buy lemonade!</t>
+          <t>At the bus stop, Lars shares some big news with Mason.
+Mom told the neighbors about his lemonade stand idea, and lots of them want to buy some!</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3824,8 +3824,8 @@
       <c r="D81" s="2" t="n"/>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Saturday morning. Lars looks at the note above his desk: 'Mountain bike'.
-His startup envelope stays at home. Today's money is just for the mall.</t>
+          <t>Saturday morning. Lars and his friends are going to the mall. Lars looks at the note and picture above his desk: 'Mountain bike'.
+He decides to leave the money for his startup at home.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -3862,8 +3862,8 @@
       <c r="D82" s="2" t="n"/>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>But today he's going to the mall with his friends.
-What he does with his money today is up to you!</t>
+          <t>Lars has two weeks of pocket money, $10, at the mall. And what he does with the money he brought, is up to you!
+Let's see the choices Lars has to make today.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -5075,7 +5075,8 @@
       <c r="E111" s="2" t="inlineStr">
         <is>
           <t>With $15 in his envelope, Lars buys a jug, cups, lemons and sugar. Mia's sign goes on the front.
-On Saturday, his stand opens by the front gate.</t>
+On Saturday, his stand opens by the front gate.
+He's one step closer to his mountain bike!</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -5096,43 +5097,6 @@
         </is>
       </c>
       <c r="K111" s="2" t="n"/>
-    </row>
-    <row r="112" ht="32" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>Scenario Beat</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="n"/>
-      <c r="D112" s="2" t="n"/>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>He's one step closer to his mountain bike!</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-lars-cheering-bike-r1.webp</t>
-        </is>
-      </c>
-      <c r="G112" s="2" t="n"/>
-      <c r="H112" s="2" t="n"/>
-      <c r="I112" s="2" t="inlineStr">
-        <is>
-          <t>After L9 S8 (beat image 2 of 2)</t>
-        </is>
-      </c>
-      <c r="J112" s="2" t="inlineStr">
-        <is>
-          <t>Lars behind his stand, proudly holding up a cup of lemonade.</t>
-        </is>
-      </c>
-      <c r="K112" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K102"/>

</xml_diff>

<commit_message>
Stage the five cleared Explorer copy cells.
Birthday money, the skin rush, the friends' ping, the gelato share, and the yo-yo question now use Cath's US spelling. The gelato beat keeps its approved still.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
+++ b/lib/academy/lessons/payload/source/explorer-m1/workbook.xlsx
@@ -741,7 +741,7 @@
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Lars's birthday money is gone. At home, he watches his big brother Senna count his money.
+          <t>Lars spent all his birthday money. At home, he watches his big brother Senna count his bills and coins.
 Senna earned it walking dogs in the neighborhood. "It's a great way to make some money," Senna says.</t>
         </is>
       </c>
@@ -787,7 +787,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Next day, Lars gets his $5 pocket money. Then his tablet flashes: 💥 RARE SKIN DEAL! ONLY 1 MINUTE LEFT! 💥 Why is the game rushing him?</t>
+          <t>The next day, Lars gets his $5 pocket money. Then his tablet flashes: 💥 RARE SKIN DEAL! ONLY 1 MINUTE LEFT! 💥 Why is the game rushing him?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1944,7 +1944,7 @@
       <c r="D36" s="2" t="n"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>At lunch, everyone's phones are buzzing. A new skin has dropped, and a countdown is ticking.
+          <t>One afternoon, Lars's friends all ping him. A new skin has dropped on their favorite game. A limited time offer and the countdown is ticking.
 Lars remembers Mason's words. His startup money is still $0.</t>
         </is>
       </c>
@@ -2833,7 +2833,7 @@
       <c r="D57" s="2" t="n"/>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Lars and Mia share the birthday gelato, one spoonful each.
+          <t>Lars and Mia share the birthday gelato. She's happy Lars came along, and Lars is grateful for Mia's generosity. He decides to repay the favor to Mia when he can.
 His startup envelope still holds $10.</t>
         </is>
       </c>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Lars has two weeks of pocket money, $10, at the mall. His startup money is safe at home. He sees a glow-in-the-dark yo-yo for $6. What do you want Lars to do?</t>
+          <t>Lars sees a glow-in-the-dark yo-yo for $6. What do you want Lars to do?</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">

</xml_diff>